<commit_message>
Día 5: Reporte de comparacion de precios en Excel
</commit_message>
<xml_diff>
--- a/src/book_manager/reportes/reporte_comparacion_precios.xlsx
+++ b/src/book_manager/reportes/reporte_comparacion_precios.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,25 +436,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Moneda</t>
+          <t>Precio interno</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Precio interno</t>
+          <t>Precio web</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Precio web</t>
+          <t>Diferencia</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Diferencia</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Fecha de extracción</t>
         </is>
@@ -466,23 +461,18 @@
           <t>El Aleph</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
+      <c r="B2" t="n">
+        <v>11200</v>
       </c>
       <c r="C2" t="n">
-        <v>11200</v>
+        <v>45499</v>
       </c>
       <c r="D2" t="n">
-        <v>45499</v>
-      </c>
-      <c r="E2" t="n">
         <v>34299</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:02</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:45:03</t>
         </is>
       </c>
     </row>
@@ -492,23 +482,18 @@
           <t>Sobre héroes y tumbas</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
+      <c r="B3" t="n">
+        <v>18.5</v>
       </c>
       <c r="C3" t="n">
-        <v>18.5</v>
+        <v>47900</v>
       </c>
       <c r="D3" t="n">
-        <v>47900</v>
-      </c>
-      <c r="E3" t="n">
         <v>47881.5</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:02</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:45:03</t>
         </is>
       </c>
     </row>
@@ -518,23 +503,18 @@
           <t>Fundación e Imperio</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
+      <c r="B4" t="n">
+        <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>15</v>
+        <v>36999</v>
       </c>
       <c r="D4" t="n">
-        <v>36999</v>
-      </c>
-      <c r="E4" t="n">
         <v>36984</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:06</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:45:06</t>
         </is>
       </c>
     </row>
@@ -544,23 +524,18 @@
           <t>Steve Jobs</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
+      <c r="B5" t="n">
+        <v>24.9</v>
       </c>
       <c r="C5" t="n">
-        <v>24.9</v>
+        <v>46499</v>
       </c>
       <c r="D5" t="n">
-        <v>46499</v>
-      </c>
-      <c r="E5" t="n">
         <v>46474.1</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:16</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:45:16</t>
         </is>
       </c>
     </row>
@@ -570,75 +545,39 @@
           <t>El poder del ahora</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
+      <c r="B6" t="n">
+        <v>16750</v>
       </c>
       <c r="C6" t="n">
-        <v>16750</v>
+        <v>33999</v>
       </c>
       <c r="D6" t="n">
-        <v>33999</v>
-      </c>
-      <c r="E6" t="n">
         <v>17249</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:15</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:45:13</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>La sombra del viento</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
+          <t>historia del tiempo</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>19800</v>
       </c>
       <c r="C7" t="n">
-        <v>21</v>
+        <v>37900</v>
       </c>
       <c r="D7" t="n">
-        <v>44900</v>
-      </c>
-      <c r="E7" t="n">
-        <v>44879</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>historia del tiempo</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ARS</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>19800</v>
-      </c>
-      <c r="D8" t="n">
-        <v>37900</v>
-      </c>
-      <c r="E8" t="n">
         <v>18100</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-10-25T00:24:20</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-10-25T15:45:19</t>
         </is>
       </c>
     </row>

</xml_diff>